<commit_message>
Lancement du pipe sur la donnée par défaut
</commit_message>
<xml_diff>
--- a/templates/Benchmark Marché/master.xlsx
+++ b/templates/Benchmark Marché/master.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mosch\Bureau\KAIVAA\kaivaa-builder\templates\Fiche d'identité des entreprises\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mosch\Bureau\KAIVAA\kaivaa-builder\templates\Benchmark Marché\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2BC591E-DBBD-47F0-8B0F-63361337E1FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E40CA923-E9FA-42F1-AD89-02249666D090}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4155" yWindow="4155" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="6" xr2:uid="{1FFF5854-B54B-4C80-B65C-C43C5EF7384C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{1FFF5854-B54B-4C80-B65C-C43C5EF7384C}"/>
   </bookViews>
   <sheets>
     <sheet name="DONNÉES BRUTES" sheetId="26" r:id="rId1"/>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="164">
   <si>
     <t>Marque</t>
   </si>
@@ -201,9 +201,6 @@
   </si>
   <si>
     <t>confidentiality</t>
-  </si>
-  <si>
-    <t>Entreprises.Nom</t>
   </si>
   <si>
     <t>Public</t>
@@ -470,12 +467,6 @@
     <t>[Segment]</t>
   </si>
   <si>
-    <t>Entreprises.Activité</t>
-  </si>
-  <si>
-    <t>Entreprises.Activité détaillée</t>
-  </si>
-  <si>
     <t>19,46</t>
   </si>
   <si>
@@ -564,6 +555,18 @@
   </si>
   <si>
     <t>résultat net</t>
+  </si>
+  <si>
+    <t>Code_NACE</t>
+  </si>
+  <si>
+    <t>Nom_de_l'entreprise</t>
+  </si>
+  <si>
+    <t>Groupes_(NACE3)</t>
+  </si>
+  <si>
+    <t>Classe_(NACE4)</t>
   </si>
 </sst>
 </file>
@@ -20732,9 +20735,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{79E1CCFD-C29F-4239-8558-4F70F8B05FAD}" name="Performance" displayName="Performance" ref="A1:Z2" totalsRowShown="0">
-  <autoFilter ref="A1:Z2" xr:uid="{79E1CCFD-C29F-4239-8558-4F70F8B05FAD}"/>
-  <tableColumns count="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{79E1CCFD-C29F-4239-8558-4F70F8B05FAD}" name="Performance" displayName="Performance" ref="A1:AA2" totalsRowShown="0">
+  <autoFilter ref="A1:AA2" xr:uid="{79E1CCFD-C29F-4239-8558-4F70F8B05FAD}"/>
+  <tableColumns count="27">
     <tableColumn id="1" xr3:uid="{D9C00F17-D0B9-47E9-BDD3-4D9C5C0FDED0}" name="siren"/>
     <tableColumn id="2" xr3:uid="{72D0A89F-A76F-4AC4-9D3A-4CD3F1A55A5C}" name="date_cloture_exercice" dataDxfId="28"/>
     <tableColumn id="3" xr3:uid="{3EFD615F-AA2D-459F-B4C7-CFFC22318CC1}" name="Chiffre_d_affaires"/>
@@ -20758,9 +20761,10 @@
     <tableColumn id="21" xr3:uid="{67FEC185-0EAF-4CAF-A9E3-D005531B61AC}" name="Credit_fournisseurs_Jours" dataDxfId="14"/>
     <tableColumn id="22" xr3:uid="{AF3E4C10-4D82-4995-9FFA-7E2CE8CB46A2}" name="type_bilan" dataDxfId="13"/>
     <tableColumn id="23" xr3:uid="{465A446E-7698-4C88-BB95-D9C31EA7A990}" name="confidentiality" dataDxfId="12"/>
-    <tableColumn id="24" xr3:uid="{7E0EE648-DC7A-4C10-AE55-84039A393AD9}" name="Entreprises.Nom" dataDxfId="11"/>
-    <tableColumn id="25" xr3:uid="{03B03CBA-639B-4937-9583-2135A393ADA7}" name="Entreprises.Activité"/>
-    <tableColumn id="26" xr3:uid="{011A9113-0055-4B4B-9BB8-F00CE3094B88}" name="Entreprises.Activité détaillée"/>
+    <tableColumn id="24" xr3:uid="{7E0EE648-DC7A-4C10-AE55-84039A393AD9}" name="Nom_de_l'entreprise" dataDxfId="11"/>
+    <tableColumn id="27" xr3:uid="{21699414-72C7-4A4E-94EA-765FF08C8A28}" name="Code_NACE"/>
+    <tableColumn id="25" xr3:uid="{03B03CBA-639B-4937-9583-2135A393ADA7}" name="Groupes_(NACE3)"/>
+    <tableColumn id="26" xr3:uid="{011A9113-0055-4B4B-9BB8-F00CE3094B88}" name="Classe_(NACE4)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -21030,7 +21034,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF961E35-3C9A-4571-868D-430D15168DE6}">
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AA2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -21057,11 +21061,12 @@
     <col min="22" max="22" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="28" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="80.88671875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="66.109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="56.21875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="80.88671875" customWidth="1"/>
+    <col min="26" max="26" width="66.109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="56.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>19</v>
       </c>
@@ -21132,16 +21137,19 @@
         <v>41</v>
       </c>
       <c r="X1" t="s">
-        <v>42</v>
+        <v>161</v>
       </c>
       <c r="Y1" t="s">
-        <v>131</v>
+        <v>160</v>
       </c>
       <c r="Z1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
+        <v>162</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>476480330</v>
       </c>
@@ -21170,7 +21178,7 @@
         <v>48635</v>
       </c>
       <c r="J2" s="38" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="K2" s="38">
         <v>-1111</v>
@@ -21185,7 +21193,7 @@
         <v>-12127</v>
       </c>
       <c r="O2" s="38" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="P2" s="38">
         <v>-9344</v>
@@ -21209,16 +21217,16 @@
         <v>10</v>
       </c>
       <c r="W2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="X2" t="s">
-        <v>87</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="Z2" t="s">
-        <v>86</v>
+        <v>82</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -21272,16 +21280,16 @@
         <v>11</v>
       </c>
       <c r="D10" s="41" t="s">
+        <v>126</v>
+      </c>
+      <c r="E10" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="E10" s="42" t="s">
-        <v>128</v>
-      </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
@@ -21290,19 +21298,19 @@
         <v>1</v>
       </c>
       <c r="B11" s="43" cm="1">
-        <f t="array" ref="B11">_xlfn.UNIQUE(Performance[siren])</f>
+        <f t="array" ref="B11">_xlfn.UNIQUE(_xlfn.SORTBY(Performance[siren],Performance[Chiffre_d_affaires],-1))</f>
         <v>476480330</v>
       </c>
       <c r="C11" s="44" t="str" cm="1">
-        <f t="array" ref="C11">INDEX(Performance[Entreprises.Nom],MATCH(_xlfn.ANCHORARRAY($B$11),Performance[siren],0))</f>
+        <f t="array" ref="C11">INDEX(Performance[Nom_de_l''entreprise],MATCH(_xlfn.ANCHORARRAY($B$11),Performance[siren],0))</f>
         <v>LUTTI</v>
       </c>
       <c r="D11" s="44" t="str" cm="1">
-        <f t="array" ref="D11">INDEX(Performance[Entreprises.Activité],MATCH(_xlfn.ANCHORARRAY($B$11),Performance[siren],0))</f>
+        <f t="array" ref="D11">INDEX(Performance[Groupes_(NACE3)],MATCH(_xlfn.ANCHORARRAY($B$11),Performance[siren],0))</f>
         <v>Fabrication d'autres produits alimentaires</v>
       </c>
       <c r="E11" s="44" t="str" cm="1">
-        <f t="array" ref="E11">INDEX(Performance[Entreprises.Activité détaillée],MATCH(_xlfn.ANCHORARRAY($B$11),Performance[siren],0))</f>
+        <f t="array" ref="E11">INDEX(Performance[Classe_(NACE4)],MATCH(_xlfn.ANCHORARRAY($B$11),Performance[siren],0))</f>
         <v>Fabrication de cacao, chocolat et de produits de confiserie</v>
       </c>
       <c r="F11" cm="1">
@@ -21310,7 +21318,7 @@
         <v>64657526</v>
       </c>
       <c r="H11" s="21" cm="1">
-        <f t="array" ref="H11">_xlfn.SORTBY(_xlfn._xlws.FILTER(Performance[date_cloture_exercice],Performance[Entreprises.Nom]=Entreprise),_xlfn._xlws.FILTER(Performance[date_cloture_exercice],Performance[Entreprises.Nom]=Entreprise),1)</f>
+        <f t="array" ref="H11">_xlfn.SORTBY(_xlfn._xlws.FILTER(Performance[date_cloture_exercice],Performance[Nom_de_l''entreprise]=Entreprise),_xlfn._xlws.FILTER(Performance[date_cloture_exercice],Performance[Nom_de_l''entreprise]=Entreprise),1)</f>
         <v>44196</v>
       </c>
     </row>
@@ -27370,442 +27378,442 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" t="s">
         <v>127</v>
       </c>
-      <c r="B1" t="s">
-        <v>128</v>
-      </c>
       <c r="C1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" t="s">
         <v>79</v>
       </c>
-      <c r="B2" t="s">
-        <v>80</v>
-      </c>
       <c r="C2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" t="s">
         <v>83</v>
       </c>
-      <c r="B5" t="s">
-        <v>84</v>
-      </c>
       <c r="C5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C6" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C7" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C8" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C9" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C10" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B12" t="s">
         <v>92</v>
       </c>
-      <c r="B12" t="s">
-        <v>93</v>
-      </c>
       <c r="C12" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C13" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C14" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C15" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C16" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C17" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C18" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C19" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>100</v>
+      </c>
+      <c r="B20" t="s">
         <v>101</v>
       </c>
-      <c r="B20" t="s">
-        <v>102</v>
-      </c>
       <c r="C20" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B21" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C21" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C22" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B23" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C23" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B24" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C24" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
+        <v>106</v>
+      </c>
+      <c r="B25" t="s">
         <v>107</v>
       </c>
-      <c r="B25" t="s">
-        <v>108</v>
-      </c>
       <c r="C25" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B26" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C26" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B27" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C27" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B28" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C28" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C29" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
+        <v>112</v>
+      </c>
+      <c r="B30" t="s">
         <v>113</v>
       </c>
-      <c r="B30" t="s">
-        <v>114</v>
-      </c>
       <c r="C30" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B31" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C31" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B32" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B33" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C33" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
+        <v>117</v>
+      </c>
+      <c r="B34" t="s">
         <v>118</v>
       </c>
-      <c r="B34" t="s">
-        <v>119</v>
-      </c>
       <c r="C34" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B35" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C35" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B36" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C36" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B37" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C37" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
+        <v>122</v>
+      </c>
+      <c r="B38" t="s">
         <v>123</v>
       </c>
-      <c r="B38" t="s">
-        <v>124</v>
-      </c>
       <c r="C38" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B39" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C39" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B40" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C40" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -27847,10 +27855,10 @@
     </row>
     <row r="5" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C5" s="37" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E5" s="37" t="str">
         <f>IF(OR(Balises!$E$8&gt;=1,Balises!$E$9&gt;=1),Balises!$E$2,"")</f>
@@ -27871,19 +27879,19 @@
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C7" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="D7" s="12" t="s">
-        <v>56</v>
-      </c>
       <c r="E7" s="29">
-        <f>INDEX(Performance[siren],MATCH(Entreprise,Performance[Entreprises.Nom],0))</f>
+        <f>INDEX(Performance[siren],MATCH(Entreprise,Performance[Nom_de_l''entreprise],0))</f>
         <v>476480330</v>
       </c>
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C8" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>23</v>
@@ -27895,10 +27903,10 @@
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C9" s="12" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E9" s="27">
         <f>Analyse!$AA$5</f>
@@ -27907,22 +27915,22 @@
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C10" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E10" s="26">
-        <f>SUMIFS(Performance[Resultat_net],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],Analyse!$E$3)</f>
+        <f>SUMIFS(Performance[Resultat_net],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],Analyse!$E$3)</f>
         <v>-2924242</v>
       </c>
     </row>
     <row r="11" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C11" s="12" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E11" s="26">
         <f>INDEX(_xlfn.ANCHORARRAY(Analyse!$C$7),MATCH($E$15,_xlfn.ANCHORARRAY(Analyse!$E$7),0))</f>
@@ -27931,10 +27939,10 @@
     </row>
     <row r="12" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C12" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E12" s="31" t="str">
         <f>Analyse!$G$4</f>
@@ -27943,10 +27951,10 @@
     </row>
     <row r="13" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C13" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E13" s="31" t="str">
         <f>Analyse!$R$4</f>
@@ -27955,10 +27963,10 @@
     </row>
     <row r="14" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C14" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E14" s="32">
         <f>MIN(_xlfn.ANCHORARRAY(Analyse!$E$7))</f>
@@ -27967,10 +27975,10 @@
     </row>
     <row r="15" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C15" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E15" s="32">
         <f>MAX(_xlfn.ANCHORARRAY(Analyse!$E$7))</f>
@@ -27979,27 +27987,27 @@
     </row>
     <row r="16" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C16" s="12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="32" t="str">
-        <f>INDEX(Performance[Entreprises.Activité],MATCH(siren,Performance[siren],0))</f>
+        <f>INDEX(Performance[Groupes_(NACE3)],MATCH(siren,Performance[siren],0))</f>
         <v>Fabrication d'autres produits alimentaires</v>
       </c>
     </row>
     <row r="17" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C17" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="32" t="str">
-        <f>INDEX(Performance[Entreprises.Activité détaillée],MATCH(siren,Performance[siren],0))</f>
+        <f>INDEX(Performance[Classe_(NACE4)],MATCH(siren,Performance[siren],0))</f>
         <v>Fabrication de cacao, chocolat et de produits de confiserie</v>
       </c>
     </row>
     <row r="18" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C18" s="12" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D18" s="12"/>
       <c r="E18" s="32" t="str">
@@ -28012,11 +28020,11 @@
         <v>5</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E19" s="20">
         <f ca="1">TODAY()</f>
-        <v>45935</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="20" spans="3:5" x14ac:dyDescent="0.35">
@@ -28064,7 +28072,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.35">
@@ -28072,7 +28080,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.35">
@@ -28176,16 +28184,16 @@
         <v>-6041459</v>
       </c>
       <c r="AH3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ3" t="s">
         <v>73</v>
       </c>
-      <c r="AI3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AJ3" t="s">
+      <c r="AK3" t="s">
         <v>74</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="4" spans="2:37" x14ac:dyDescent="0.4">
@@ -28214,11 +28222,11 @@
         <v>NA</v>
       </c>
       <c r="Z4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA4" s="33">
-        <f>SUMIFS(Performance[EBE],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],$E$3)/
-SUMIFS(Performance[Chiffre_d_affaires],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
+        <f>SUMIFS(Performance[EBE],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],$E$3)/
+SUMIFS(Performance[Chiffre_d_affaires],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
         <v>-9.3437831196943724E-2</v>
       </c>
       <c r="AB4" s="30">
@@ -28226,10 +28234,10 @@
         <v>1.0934378311969437</v>
       </c>
       <c r="AE4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AF4" s="28">
-        <f>SUMIFS(Performance[Chiffre_d_affaires],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
+        <f>SUMIFS(Performance[Chiffre_d_affaires],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
         <v>64657526</v>
       </c>
       <c r="AG4" s="35">
@@ -28243,11 +28251,11 @@
     </row>
     <row r="5" spans="2:37" x14ac:dyDescent="0.4">
       <c r="Z5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA5" s="33">
-        <f>SUMIFS(Performance[Resultat_net],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],$E$3)/
-SUMIFS(Performance[Chiffre_d_affaires],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
+        <f>SUMIFS(Performance[Resultat_net],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],$E$3)/
+SUMIFS(Performance[Chiffre_d_affaires],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
         <v>-4.5226629920854071E-2</v>
       </c>
       <c r="AB5" s="30">
@@ -28255,7 +28263,7 @@
         <v>1.0452266299208541</v>
       </c>
       <c r="AE5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AF5" s="28">
         <f>AF6-AF4</f>
@@ -28280,71 +28288,71 @@
     </row>
     <row r="6" spans="2:37" x14ac:dyDescent="0.4">
       <c r="B6" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="D6" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="E6" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="F6" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="F6" s="26" t="s">
+      <c r="G6" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="G6" s="24" t="s">
+      <c r="H6" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="I6" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="J6" s="24" t="s">
         <v>51</v>
-      </c>
-      <c r="H6" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="I6" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="J6" s="24" t="s">
-        <v>52</v>
       </c>
       <c r="K6" s="24"/>
       <c r="M6" s="25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N6" s="26" t="s">
         <v>23</v>
       </c>
       <c r="O6" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="P6" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="P6" s="24" t="s">
+      <c r="Q6" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="Q6" s="26" t="s">
+      <c r="R6" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="R6" s="24" t="s">
+      <c r="S6" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="T6" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="U6" s="24" t="s">
         <v>51</v>
-      </c>
-      <c r="S6" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="T6" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="U6" s="24" t="s">
-        <v>52</v>
       </c>
       <c r="V6" s="24" t="s">
         <v>23</v>
       </c>
       <c r="W6" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AE6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AF6" s="28">
-        <f>SUMIFS(Performance[Marge_brute],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
+        <f>SUMIFS(Performance[Marge_brute],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
         <v>34888091</v>
       </c>
       <c r="AG6" s="35">
@@ -28363,7 +28371,7 @@
         <v>44196</v>
       </c>
       <c r="C7" s="26" cm="1">
-        <f t="array" ref="C7">SUMIFS(Performance[Chiffre_d_affaires],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],_xlfn.ANCHORARRAY($B7))</f>
+        <f t="array" ref="C7">SUMIFS(Performance[Chiffre_d_affaires],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],_xlfn.ANCHORARRAY($B7))</f>
         <v>64657526</v>
       </c>
       <c r="D7" s="24" cm="1">
@@ -28401,7 +28409,7 @@
         <v>44196</v>
       </c>
       <c r="N7" s="26" cm="1">
-        <f t="array" ref="N7">SUMIFS(Performance[EBE],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],_xlfn.ANCHORARRAY($B7))</f>
+        <f t="array" ref="N7">SUMIFS(Performance[EBE],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],_xlfn.ANCHORARRAY($B7))</f>
         <v>-6041459</v>
       </c>
       <c r="O7" s="24" cm="1">
@@ -28434,7 +28442,7 @@
         <v>-</v>
       </c>
       <c r="V7" s="28" cm="1">
-        <f t="array" ref="V7">SUMIFS(Performance[EBE],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],_xlfn.ANCHORARRAY($B7))</f>
+        <f t="array" ref="V7">SUMIFS(Performance[EBE],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],_xlfn.ANCHORARRAY($B7))</f>
         <v>-6041459</v>
       </c>
       <c r="W7" s="3" cm="1">
@@ -28442,7 +28450,7 @@
         <v>-9.3437831196943724E-2</v>
       </c>
       <c r="AE7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AF7" s="28">
         <f>AF8-AF6</f>
@@ -28486,7 +28494,7 @@
         <v>23</v>
       </c>
       <c r="AF8" s="28">
-        <f>SUMIFS(Performance[EBE],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
+        <f>SUMIFS(Performance[EBE],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
         <v>-6041459</v>
       </c>
       <c r="AG8" s="35">
@@ -28517,7 +28525,7 @@
       <c r="T9" s="24"/>
       <c r="V9" s="28"/>
       <c r="AE9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AF9" s="28">
         <f>AF10-AF8</f>
@@ -28558,10 +28566,10 @@
       <c r="T10" s="24"/>
       <c r="V10" s="28"/>
       <c r="AE10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AF10" s="28">
-        <f>SUMIFS(Performance[Resultat_net],Performance[Entreprises.Nom],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
+        <f>SUMIFS(Performance[Resultat_net],Performance[Nom_de_l''entreprise],Entreprise,Performance[date_cloture_exercice],$E$3)</f>
         <v>-2924242</v>
       </c>
       <c r="AG10" s="35">

</xml_diff>

<commit_message>
Sécurisation boc code 1
</commit_message>
<xml_diff>
--- a/templates/Benchmark Marché/master.xlsx
+++ b/templates/Benchmark Marché/master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mosch\Bureau\KAIVAA\kaivaa-builder\templates\Benchmark Marché\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{840F9717-6E37-4845-80A7-5C4F50DB8682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5218DEF-AD1A-4904-9599-FC609AC610F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11295" activeTab="5" xr2:uid="{1FFF5854-B54B-4C80-B65C-C43C5EF7384C}"/>
+    <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11295" activeTab="6" xr2:uid="{1FFF5854-B54B-4C80-B65C-C43C5EF7384C}"/>
   </bookViews>
   <sheets>
     <sheet name="DONNÉES BRUTES" sheetId="26" r:id="rId1"/>
@@ -21312,7 +21312,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="43" cm="1">
-        <f t="array" ref="B11">_xlfn.UNIQUE(_xlfn.SORTBY(Performance[siren],Performance[Chiffre_d_affaires],-1))</f>
+        <f t="array" ref="B11">_xlfn.UNIQUE(_xlfn._xlws.FILTER(_xlfn.SORTBY(Performance[siren],Performance[Chiffre_d_affaires],-1),_xlfn.SORTBY(Performance[Chiffre_d_affaires],Performance[Chiffre_d_affaires],-1)&gt;3000000))</f>
         <v>476480330</v>
       </c>
       <c r="C11" s="44" t="str" cm="1">
@@ -28131,7 +28131,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="17">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="E6" s="15" t="str" cm="1">
         <f t="array" ref="E6">INDEX(Listes!$C$11:$C$676,Loop[[#This Row],[Itération]])</f>

</xml_diff>